<commit_message>
add state election term variable to more datasets and added links to ppg and cabinet data from statepol
</commit_message>
<xml_diff>
--- a/inst/extdata/coldesc.xlsx
+++ b/inst/extdata/coldesc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10905"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rober\Desktop\add\bundeslaendeR\inst\extdata\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertstelzle/git_projekte/bundeslaendeR/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84423A52-3BA8-486B-AB17-3F933C7F9CE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C733AC73-CC20-C348-88E8-4956D76FE702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="2655" windowWidth="25440" windowHeight="15390" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="21300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
   <si>
     <t>colname</t>
   </si>
@@ -536,6 +536,36 @@
   </si>
   <si>
     <t>ZA Dataset ID</t>
+  </si>
+  <si>
+    <t>landtag_state_abb</t>
+  </si>
+  <si>
+    <t>electoralperiod</t>
+  </si>
+  <si>
+    <t>ppg</t>
+  </si>
+  <si>
+    <t>link_notes</t>
+  </si>
+  <si>
+    <t>Notes on link</t>
+  </si>
+  <si>
+    <t>cabinet</t>
+  </si>
+  <si>
+    <t>Name of cabinet in StatePol data</t>
+  </si>
+  <si>
+    <t>Name of Parliamentary Party Group in StatePol data</t>
+  </si>
+  <si>
+    <t>State abbreviation in StatePol data</t>
+  </si>
+  <si>
+    <t>State election term in StatePol data</t>
   </si>
 </sst>
 </file>
@@ -888,14 +918,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B86"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:B91"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="38.7109375" customWidth="1"/>
-    <col min="2" max="2" width="67.7109375" customWidth="1"/>
+    <col min="1" max="1" width="38.6640625" customWidth="1"/>
+    <col min="2" max="2" width="67.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -903,7 +933,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -911,7 +941,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -919,7 +949,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -927,7 +957,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -935,7 +965,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -943,7 +973,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -951,7 +981,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -959,7 +989,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>151</v>
       </c>
@@ -967,7 +997,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -975,7 +1005,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -983,7 +1013,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -991,7 +1021,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -999,7 +1029,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1007,7 +1037,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1015,7 +1045,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1023,7 +1053,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1031,7 +1061,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1039,7 +1069,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1047,7 +1077,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1055,7 +1085,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1063,7 +1093,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1071,7 +1101,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1079,7 +1109,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1087,7 +1117,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1095,7 +1125,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1103,7 +1133,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1111,7 +1141,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1119,7 +1149,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1127,7 +1157,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1135,7 +1165,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1143,7 +1173,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1151,7 +1181,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1159,7 +1189,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1167,7 +1197,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1175,7 +1205,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1183,7 +1213,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1191,7 +1221,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -1199,7 +1229,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1207,7 +1237,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>38</v>
       </c>
@@ -1215,7 +1245,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -1223,7 +1253,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -1231,7 +1261,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>41</v>
       </c>
@@ -1239,7 +1269,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>42</v>
       </c>
@@ -1247,7 +1277,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -1255,7 +1285,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -1263,7 +1293,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -1271,7 +1301,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>46</v>
       </c>
@@ -1279,7 +1309,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -1287,7 +1317,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -1295,7 +1325,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>49</v>
       </c>
@@ -1303,7 +1333,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -1311,7 +1341,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>51</v>
       </c>
@@ -1319,7 +1349,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>52</v>
       </c>
@@ -1327,7 +1357,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>53</v>
       </c>
@@ -1335,7 +1365,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -1343,7 +1373,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>55</v>
       </c>
@@ -1351,7 +1381,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>56</v>
       </c>
@@ -1359,7 +1389,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>57</v>
       </c>
@@ -1367,7 +1397,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>58</v>
       </c>
@@ -1375,7 +1405,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>59</v>
       </c>
@@ -1383,7 +1413,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>60</v>
       </c>
@@ -1391,7 +1421,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>61</v>
       </c>
@@ -1399,7 +1429,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>62</v>
       </c>
@@ -1407,7 +1437,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -1415,7 +1445,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>64</v>
       </c>
@@ -1423,7 +1453,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>65</v>
       </c>
@@ -1431,7 +1461,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>66</v>
       </c>
@@ -1439,7 +1469,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>67</v>
       </c>
@@ -1447,7 +1477,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>68</v>
       </c>
@@ -1455,7 +1485,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>69</v>
       </c>
@@ -1463,7 +1493,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>70</v>
       </c>
@@ -1471,7 +1501,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -1479,7 +1509,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>72</v>
       </c>
@@ -1487,7 +1517,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -1495,7 +1525,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>74</v>
       </c>
@@ -1503,7 +1533,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>152</v>
       </c>
@@ -1511,7 +1541,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>153</v>
       </c>
@@ -1519,7 +1549,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>156</v>
       </c>
@@ -1527,7 +1557,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>158</v>
       </c>
@@ -1535,7 +1565,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>161</v>
       </c>
@@ -1543,7 +1573,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>162</v>
       </c>
@@ -1551,7 +1581,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>164</v>
       </c>
@@ -1559,7 +1589,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>165</v>
       </c>
@@ -1567,7 +1597,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>166</v>
       </c>
@@ -1575,12 +1605,52 @@
         <v>170</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>167</v>
       </c>
       <c r="B86" t="s">
         <v>171</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" t="s">
+        <v>172</v>
+      </c>
+      <c r="B87" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>173</v>
+      </c>
+      <c r="B88" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>174</v>
+      </c>
+      <c r="B89" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>175</v>
+      </c>
+      <c r="B90" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>177</v>
+      </c>
+      <c r="B91" t="s">
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
add normalized gallaghar disprop index fix test warning fix codebook typo fix rbuildignore warnings
</commit_message>
<xml_diff>
--- a/inst/extdata/coldesc.xlsx
+++ b/inst/extdata/coldesc.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10905"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/robertstelzle/git_projekte/bundeslaendeR/inst/extdata/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au785183\git_projects\bundeslaendeR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C733AC73-CC20-C348-88E8-4956D76FE702}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A96001-445C-465B-876A-976BFA3859CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="21300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
   <si>
     <t>colname</t>
   </si>
@@ -566,6 +566,12 @@
   </si>
   <si>
     <t>State election term in StatePol data</t>
+  </si>
+  <si>
+    <t>disprop_gallagher_normalized</t>
+  </si>
+  <si>
+    <t>Gallagher index of electoral disproportionality, normalized by effective number of parties (Bailey 2026).</t>
   </si>
 </sst>
 </file>
@@ -616,7 +622,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -918,14 +924,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B91"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B92"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="38.6640625" customWidth="1"/>
-    <col min="2" max="2" width="67.6640625" customWidth="1"/>
+    <col min="1" max="1" width="38.7109375" customWidth="1"/>
+    <col min="2" max="2" width="67.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -933,7 +939,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -941,7 +947,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -949,7 +955,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -957,7 +963,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -965,7 +971,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -973,7 +979,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -981,7 +987,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -989,7 +995,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>151</v>
       </c>
@@ -997,7 +1003,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1005,7 +1011,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -1013,7 +1019,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -1021,7 +1027,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -1029,7 +1035,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>12</v>
       </c>
@@ -1037,7 +1043,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -1045,7 +1051,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -1053,7 +1059,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -1061,7 +1067,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -1069,7 +1075,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -1077,7 +1083,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -1085,7 +1091,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -1093,7 +1099,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -1101,7 +1107,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -1109,7 +1115,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>22</v>
       </c>
@@ -1117,7 +1123,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>23</v>
       </c>
@@ -1125,7 +1131,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>24</v>
       </c>
@@ -1133,7 +1139,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>25</v>
       </c>
@@ -1141,7 +1147,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>26</v>
       </c>
@@ -1149,7 +1155,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>27</v>
       </c>
@@ -1157,7 +1163,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>28</v>
       </c>
@@ -1165,7 +1171,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>29</v>
       </c>
@@ -1173,7 +1179,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>30</v>
       </c>
@@ -1181,7 +1187,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>31</v>
       </c>
@@ -1189,7 +1195,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>32</v>
       </c>
@@ -1197,7 +1203,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>33</v>
       </c>
@@ -1205,7 +1211,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>34</v>
       </c>
@@ -1213,7 +1219,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>35</v>
       </c>
@@ -1221,7 +1227,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>36</v>
       </c>
@@ -1229,7 +1235,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -1237,7 +1243,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>38</v>
       </c>
@@ -1245,7 +1251,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -1253,7 +1259,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>40</v>
       </c>
@@ -1261,7 +1267,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>41</v>
       </c>
@@ -1269,7 +1275,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>42</v>
       </c>
@@ -1277,7 +1283,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -1285,7 +1291,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -1293,7 +1299,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -1301,7 +1307,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>46</v>
       </c>
@@ -1309,7 +1315,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>47</v>
       </c>
@@ -1317,7 +1323,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>48</v>
       </c>
@@ -1325,7 +1331,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>49</v>
       </c>
@@ -1333,7 +1339,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>50</v>
       </c>
@@ -1341,7 +1347,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>51</v>
       </c>
@@ -1349,7 +1355,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>52</v>
       </c>
@@ -1357,7 +1363,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>53</v>
       </c>
@@ -1365,7 +1371,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>54</v>
       </c>
@@ -1373,7 +1379,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>55</v>
       </c>
@@ -1381,7 +1387,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>56</v>
       </c>
@@ -1389,7 +1395,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>57</v>
       </c>
@@ -1397,7 +1403,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>58</v>
       </c>
@@ -1405,7 +1411,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>59</v>
       </c>
@@ -1413,7 +1419,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>60</v>
       </c>
@@ -1421,7 +1427,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>61</v>
       </c>
@@ -1429,7 +1435,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>62</v>
       </c>
@@ -1437,7 +1443,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>63</v>
       </c>
@@ -1445,7 +1451,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>64</v>
       </c>
@@ -1453,7 +1459,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>65</v>
       </c>
@@ -1461,7 +1467,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>66</v>
       </c>
@@ -1469,7 +1475,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>67</v>
       </c>
@@ -1477,7 +1483,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>68</v>
       </c>
@@ -1485,7 +1491,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>69</v>
       </c>
@@ -1493,7 +1499,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>70</v>
       </c>
@@ -1501,7 +1507,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -1509,7 +1515,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>72</v>
       </c>
@@ -1517,7 +1523,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -1525,7 +1531,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>74</v>
       </c>
@@ -1533,7 +1539,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>152</v>
       </c>
@@ -1541,7 +1547,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>153</v>
       </c>
@@ -1549,7 +1555,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>156</v>
       </c>
@@ -1557,7 +1563,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>158</v>
       </c>
@@ -1565,7 +1571,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>161</v>
       </c>
@@ -1573,7 +1579,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>162</v>
       </c>
@@ -1581,7 +1587,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>164</v>
       </c>
@@ -1589,7 +1595,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>165</v>
       </c>
@@ -1597,7 +1603,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>166</v>
       </c>
@@ -1605,7 +1611,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>167</v>
       </c>
@@ -1613,7 +1619,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>172</v>
       </c>
@@ -1621,7 +1627,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>173</v>
       </c>
@@ -1629,7 +1635,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>174</v>
       </c>
@@ -1637,7 +1643,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>175</v>
       </c>
@@ -1645,12 +1651,20 @@
         <v>176</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>177</v>
       </c>
       <c r="B91" t="s">
         <v>178</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>182</v>
+      </c>
+      <c r="B92" t="s">
+        <v>183</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
adding link to stateparl data on parliamentary speeches
</commit_message>
<xml_diff>
--- a/inst/extdata/coldesc.xlsx
+++ b/inst/extdata/coldesc.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\au785183\git_projects\bundeslaendeR\inst\extdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09A96001-445C-465B-876A-976BFA3859CC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1871A76-D340-427A-B5F4-6B3908253DDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="190">
   <si>
     <t>colname</t>
   </si>
@@ -572,6 +572,24 @@
   </si>
   <si>
     <t>Gallagher index of electoral disproportionality, normalized by effective number of parties (Bailey 2026).</t>
+  </si>
+  <si>
+    <t>period</t>
+  </si>
+  <si>
+    <t>affiliation</t>
+  </si>
+  <si>
+    <t>Party affiliation in StateParl</t>
+  </si>
+  <si>
+    <t>Electoral period in StateParl</t>
+  </si>
+  <si>
+    <t>state_bundeslaender</t>
+  </si>
+  <si>
+    <t>State abbreviation in bundeslaendeR data</t>
   </si>
 </sst>
 </file>
@@ -924,7 +942,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B92"/>
+  <dimension ref="A1:B95"/>
   <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.7109375" customWidth="1"/>
@@ -1667,6 +1685,30 @@
         <v>183</v>
       </c>
     </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>184</v>
+      </c>
+      <c r="B93" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>185</v>
+      </c>
+      <c r="B94" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>188</v>
+      </c>
+      <c r="B95" t="s">
+        <v>189</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>